<commit_message>
docs(jd): 第一期 H-01~H-09 + DB 集成配套文档规则 (2026-08-22)
补提交：
- AGENTS.md (新增 H/M/L 审计规则 + 数据库底线 + Skill调度规则)
- docs/项目文档索引.xlsx (全项目文档索引自动生成)
- docs/2026-08-22_Excel总表实现说明.md (项目24 Excel 总表)
- docs/2026-08-22_H高危审计修复报告.md (第一期 H-01~H-09 修复报告)
- docs/config参数维护指南.md (config.xlsx 配置维护手册)
- docs/三店拆分方案.md (3 店平铺方案)
- docs/项目文件清单.md (项目文件清单)

背景：2026-08-22 第一期审计 + DB 集成MVP落地后未及时提交，
本 commit 把相关文档规则补齐入库，便于后续审计追溯。

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/项目文档索引.xlsx
+++ b/docs/项目文档索引.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="�� 文档总索引" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="�� 分类汇总" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="�� 文档总索引" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="�� 分类汇总" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -522,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1898,6 +1898,601 @@
       <c r="G39" s="2" t="inlineStr">
         <is>
           <t>自动入库 @ 2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="38" customHeight="1">
+      <c r="A40" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>DB_USAGE.md</t>
+        </is>
+      </c>
+      <c r="C40" s="10" t="inlineStr">
+        <is>
+          <t>文档</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>DB_USAGE.md</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>D:\CODE\trae\traespace\FYA箱包旗舰店\DB_USAGE.md</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t># 数据库集成使用说明（项目21，2026-08-14） &gt; 适用版本：main.py ≥ 5645769 &gt; 目的：将 20 个京东数据报表（Excel）持久化到本地 SQLite 数据库，支持每日自动滚动更新与缺失补录。</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>自动入库 @ 2026-08-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="38" customHeight="1">
+      <c r="A41" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>biz_config_loader.py</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>脚本</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>biz_config_loader.py</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>D:\CODE\trae\traespace\FYA箱包旗舰店\biz_config_loader.py</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t># -*- coding: utf-8 -*- """biz_config_loader.py ============================================================</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>自动入库 @ 2026-08-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="38" customHeight="1">
+      <c r="A42" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>daily_update.py</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>脚本</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>daily_update.py</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>D:\CODE\trae\traespace\FYA箱包旗舰店\daily_update.py</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t># -*- coding: utf-8 -*- daily_update.py ============================================================</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>自动入库 @ 2026-08-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="38" customHeight="1">
+      <c r="A43" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>db_utils.py</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>脚本</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>db_utils.py</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>D:\CODE\trae\traespace\FYA箱包旗舰店\db_utils.py</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t># -*- coding: utf-8 -*- db_utils.py ============================================================</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>自动入库 @ 2026-08-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="38" customHeight="1">
+      <c r="A44" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22_Excel总表实现说明.md</t>
+        </is>
+      </c>
+      <c r="C44" s="10" t="inlineStr">
+        <is>
+          <t>文档</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>docs/2026-08-22_Excel总表实现说明.md</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>D:\CODE\trae\traespace\FYA箱包旗舰店\docs\2026-08-22_Excel总表实现说明.md</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t># Excel 总表双输出实现说明（项目24） &gt; **生效时间**：2026-08-22 &gt; **作者**：Trae Agent</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>自动入库 @ 2026-08-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="38" customHeight="1">
+      <c r="A45" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22_H高危审计修复报告.md</t>
+        </is>
+      </c>
+      <c r="C45" s="10" t="inlineStr">
+        <is>
+          <t>文档</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>docs/2026-08-22_H高危审计修复报告.md</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>D:\CODE\trae\traespace\FYA箱包旗舰店\docs\2026-08-22_H高危审计修复报告.md</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t># 2026-08-22 H 高危审计修复报告 &gt; 任务背景：审计发现 9 条高危必须修复（H-01~H-09） &gt; 修复策略：禁止硬编码兜底，所有业务常量从 runtime_config 统一加载</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>自动入库 @ 2026-08-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="38" customHeight="1">
+      <c r="A46" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>config参数维护指南.md</t>
+        </is>
+      </c>
+      <c r="C46" s="10" t="inlineStr">
+        <is>
+          <t>文档</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>docs/config参数维护指南.md</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>D:\CODE\trae\traespace\FYA箱包旗舰店\docs\config参数维护指南.md</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t># config.xlsx 可调整参数维护指南（2026-08-21 新增） &gt; 本文档是**轻量日常维护**手册，与 `docs/维护手册.md`（Cookie / h5st 重抓）互补。 &gt;</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>自动入库 @ 2026-08-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="38" customHeight="1">
+      <c r="A47" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>三店拆分方案.md</t>
+        </is>
+      </c>
+      <c r="C47" s="10" t="inlineStr">
+        <is>
+          <t>文档</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>docs/三店拆分方案.md</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>D:\CODE\trae\traespace\FYA箱包旗舰店\docs\三店拆分方案.md</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t># 三店拆分方案（2026-08-21 设计稿，待用户确认后实施） ## 一、目标 - 当前 main.py 10,119 行单文件 → 拆为 4 个文件</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>自动入库 @ 2026-08-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="38" customHeight="1">
+      <c r="A48" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>项目文件清单.md</t>
+        </is>
+      </c>
+      <c r="C48" s="10" t="inlineStr">
+        <is>
+          <t>文档</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>docs/项目文件清单.md</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>D:\CODE\trae\traespace\FYA箱包旗舰店\docs\项目文件清单.md</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t># FYA箱包旗舰店 · 项目文件清单 &gt; **生成日期**：2026-08-21 &gt; **扫描范围**：`d:\CODE\trae\traespace\FYA箱包旗舰店`</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>自动入库 @ 2026-08-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="38" customHeight="1">
+      <c r="A49" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>excel_master.py</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>脚本</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>excel_master.py</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>D:\CODE\trae\traespace\FYA箱包旗舰店\excel_master.py</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t># -*- coding: utf-8 -*- """excel_master.py ============================================================</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>自动入库 @ 2026-08-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="38" customHeight="1">
+      <c r="A50" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>fill_missing.py</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>脚本</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>fill_missing.py</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>D:\CODE\trae\traespace\FYA箱包旗舰店\fill_missing.py</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t># -*- coding: utf-8 -*- fill_missing.py ============================================================</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>自动入库 @ 2026-08-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="38" customHeight="1">
+      <c r="A51" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>imap_config_loader.py</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>脚本</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>imap_config_loader.py</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>D:\CODE\trae\traespace\FYA箱包旗舰店\imap_config_loader.py</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t># -*- coding: utf-8 -*- """imap_config_loader.py ============================================================</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>自动入库 @ 2026-08-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="38" customHeight="1">
+      <c r="A52" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>FOLDER_NAME.md</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>文件夹说明</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>output/FYA箱包旗舰店/FOLDER_NAME.md</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>D:\CODE\trae\traespace\FYA箱包旗舰店\output\FYA箱包旗舰店\FOLDER_NAME.md</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t># 📂 文件夹命名说明：output ## 基本信息 | 项 | 内容 |</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>自动入库 @ 2026-08-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="38" customHeight="1">
+      <c r="A53" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>refresh_reports.py</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>脚本</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>refresh_reports.py</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>D:\CODE\trae\traespace\FYA箱包旗舰店\refresh_reports.py</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t># -*- coding: utf-8 -*- """refresh_reports.py ============================================================</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>自动入库 @ 2026-08-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="38" customHeight="1">
+      <c r="A54" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>rpa_run.py</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>脚本</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>rpa_run.py</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>D:\CODE\trae\traespace\FYA箱包旗舰店\rpa_run.py</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t># -*- coding: utf-8 -*- """多店铺数据导出手动触发入口（项目22，2026-08-17） 用户决策 2026-08-17：</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>自动入库 @ 2026-08-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="38" customHeight="1">
+      <c r="A55" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>runtime_config.py</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>脚本</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>runtime_config.py</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>D:\CODE\trae\traespace\FYA箱包旗舰店\runtime_config.py</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t># -*- coding: utf-8 -*- """runtime_config.py ============================================================</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>自动入库 @ 2026-08-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="38" customHeight="1">
+      <c r="A56" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>excel_master_unittest.py</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>脚本</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>tests/excel_master_unittest.py</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>D:\CODE\trae\traespace\FYA箱包旗舰店\tests\excel_master_unittest.py</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t># -*- coding: utf-8 -*- """excel_master 自测脚本（2026-08-22 项目24） 4 个核心场景（用户 spec 第九节）：</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>自动入库 @ 2026-08-22</t>
         </is>
       </c>
     </row>
@@ -2019,7 +2614,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
@@ -2034,7 +2629,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -2064,7 +2659,7 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>

</xml_diff>